<commit_message>
Aba numerada pelo volume da programação, quantos forem
O lote pode ter seis caixas. A aba saía numerada pela ordem em que o arquivo
foi montado, então um produto com mapa só no terceiro volume virava MAPA
CX01 — a aba mentia sobre qual caixa era. Agora o número vem do VOL da
programação: VOL 3/6 sai como MAPA CX03.

Dois volumes com o mesmo VOL no lote desempatam pelo código: aba repetida
não abre no Excel.

Volume ainda sem mapa continua fora do arquivo, mas o rodapé diz quantos
ficaram em vez de deixar o líder contar aba. A ordem passou a ser a da
programação, e o arquivo leva o número do lote, não o do primeiro volume.

O COMO USAR do modelo explica como abrir a próxima caixa: copia a aba, troca
o código em A1. Nome de aba não significa nada na importação — quem
identifica o mapa é o código da primeira linha.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KwoYv8EsJGsrY6sPoHB9c5
</commit_message>
<xml_diff>
--- a/modelo-mapa-trilhos.xlsx
+++ b/modelo-mapa-trilhos.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A45"/>
+  <dimension ref="A1:A51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="92" customWidth="1" min="1" max="1"/>
@@ -452,225 +452,261 @@
     </row>
     <row r="5"/>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>NO EXCEL</t>
-        </is>
-      </c>
-    </row>
-    <row r="7"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MAIS CAIXAS: copie a aba, troque o código em A1 e o nome da aba (MAPA CX03,</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>MAPA CX04, e por aí). O app lê quantas abas houver — quem identifica o mapa</t>
+        </is>
+      </c>
+    </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>é o código em A1, não o nome da aba.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>NO EXCEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>Linha 1        A1  o código do volume, o mesmo da programação</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">               B1  a descrição do volume — só para quem lê a planilha</t>
-        </is>
-      </c>
-    </row>
-    <row r="10"/>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Linha 2        o cabeçalho, sempre nesta ordem:</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">               TRILHO | OP | COD | DESCRIÇÃO ITEM | QTDE | COD | DESCRIÇÃO ITEM | QTDE</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">               O bloco COD/DESCRIÇÃO/QTDE repete: o primeiro é a peça, o</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">               segundo é o insumo que vai junto no trilho. Se um trilho</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">               B1  a descrição do volume — só para quem lê a planilha</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">               precisar de um terceiro, copie mais três colunas à direita.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16"/>
+          <t>Linha 2        o cabeçalho, sempre nesta ordem:</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">               TRILHO | OP | COD | DESCRIÇÃO ITEM | QTDE | COD | DESCRIÇÃO ITEM | QTDE</t>
+        </is>
+      </c>
+    </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Da linha 3     uma linha por trilho, do 1 até o último:</t>
+          <t xml:space="preserve">               O bloco COD/DESCRIÇÃO/QTDE repete: o primeiro é a peça, o</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>em diante</t>
+          <t xml:space="preserve">               segundo é o insumo que vai junto no trilho. Se um trilho</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">               TRILHO  o número, em ordem</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">               OP      a OP daquele trilho, escrita em toda linha com item</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">               precisar de um terceiro, copie mais três colunas à direita.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">               COD     o código da peça, como o ERP escreve</t>
+          <t>Da linha 3     uma linha por trilho, do 1 até o último:</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">               QTDE    quantas peças daquele código vão no trilho</t>
-        </is>
-      </c>
-    </row>
-    <row r="23"/>
+          <t>em diante</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">               TRILHO  o número, em ordem</t>
+        </is>
+      </c>
+    </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">               Trilho vazio: deixe a linha só com o número. Não apague a</t>
+          <t xml:space="preserve">               OP      a OP daquele trilho, escrita em toda linha com item</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">               linha — trilho vazio também é trilho na esteira.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26"/>
-    <row r="27">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>NO APP</t>
-        </is>
-      </c>
-    </row>
-    <row r="28"/>
+          <t xml:space="preserve">               COD     o código da peça, como o ERP escreve</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">               QTDE    quantas peças daquele código vão no trilho</t>
+        </is>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">               Trilho vazio: deixe a linha só com o número. Não apague a</t>
+        </is>
+      </c>
+    </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t xml:space="preserve">               linha — trilho vazio também é trilho na esteira.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>NO APP</t>
+        </is>
+      </c>
+    </row>
+    <row r="32"/>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>1. IMPORTAR EXCEL no rodapé e escolha este arquivo.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>2. Com o código escrito, o item entra direto. Item sem código o app procura</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   pelo texto, e pergunta em vez de chutar quando fica em dúvida.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>3. Confira o mapa na tela e toque em SALVAR MAPA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33"/>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>EXPORTAR EXCEL faz o caminho de volta: baixa o mapa que está na tela neste</t>
+          <t>2. Com o código escrito, o item entra direto. Item sem código o app procura</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>mesmo formato, uma aba por volume do lote. É por aí que se começa um produto</t>
+          <t xml:space="preserve">   pelo texto, e pergunta em vez de chutar quando fica em dúvida.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>novo — exporta o parecido, troca o que muda e importa de volta.</t>
+          <t>3. Confira o mapa na tela e toque em SALVAR MAPA.</t>
         </is>
       </c>
     </row>
     <row r="37"/>
     <row r="38">
-      <c r="A38" s="1" t="inlineStr">
-        <is>
-          <t>O MESMO MAPA PARA VÁRIAS CORES</t>
-        </is>
-      </c>
-    </row>
-    <row r="39"/>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>EXPORTAR EXCEL faz o caminho de volta: baixa o lote inteiro neste mesmo</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>formato, uma aba por volume, numerada pelo VOL da programação — o VOL 3/6</t>
+        </is>
+      </c>
+    </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Os códigos escritos aqui são de uma cor só. Para o mesmo mapa valer para as</t>
+          <t>sai como MAPA CX03. Volume ainda sem mapa fica de fora, e o app diz quantos</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>outras, crie uma aba PRODUTOS com as colunas ABA_MAPA e COD_PRODUTO, uma</t>
+          <t>foram. É por aí que se começa um produto novo: exporta o parecido, troca o</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>que muda e importa de volta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43"/>
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t>O MESMO MAPA PARA VÁRIAS CORES</t>
+        </is>
+      </c>
+    </row>
+    <row r="45"/>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Os códigos escritos aqui são de uma cor só. Para o mesmo mapa valer para as</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>outras, crie uma aba PRODUTOS com as colunas ABA_MAPA e COD_PRODUTO, uma</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>linha por cor. O app acha a mesma peça na outra cor pelo Nº que vem depois</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t>de MDP/MDF na descrição do ERP — esse número não muda de cor.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr">
         <is>
           <t>Colunas opcionais na PRODUTOS: COR, N_TRILHOS, VELOCIDADE, N_ESQUEMA.</t>
         </is>
       </c>
     </row>
-    <row r="45"/>
+    <row r="51"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>